<commit_message>
add m5 JavaScript advanced module with assignments and activities
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -35,7 +35,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +72,11 @@
         <fgColor rgb="00FFF3E0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4EC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -85,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -118,6 +123,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -485,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2193,6 +2204,681 @@
       <c r="E63" s="11" t="inlineStr">
         <is>
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m4/activities/lesson-24/real-time-application-using-js.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 25 – Brief on JS</t>
+        </is>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
+        <is>
+          <t>print-random-numbers</t>
+        </is>
+      </c>
+      <c r="E64" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/print-random-numbers/print-random-numbers.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C65" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 26 – Classes</t>
+        </is>
+      </c>
+      <c r="D65" s="12" t="inlineStr">
+        <is>
+          <t>class-in-js</t>
+        </is>
+      </c>
+      <c r="E65" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/class-in-js/class-in-js.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 27 – Array Sorting &amp; Mapping</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
+        <is>
+          <t>map-and-arrange-an-array</t>
+        </is>
+      </c>
+      <c r="E66" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/map-and-arrange-an-array/map-and-arrange-an-array.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C67" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 28 – JS in Detail</t>
+        </is>
+      </c>
+      <c r="D67" s="12" t="inlineStr">
+        <is>
+          <t>handle-errors-in-js</t>
+        </is>
+      </c>
+      <c r="E67" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/handle-errors-in-js/handle-errors-in-js.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="12" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C68" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 29 – JSON &amp; Async</t>
+        </is>
+      </c>
+      <c r="D68" s="12" t="inlineStr">
+        <is>
+          <t>asynchronous-functions-in-js</t>
+        </is>
+      </c>
+      <c r="E68" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/asynchronous-functions-in-js/asynchronous-functions-in-js.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 25 – Brief on JS</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>data-types-in-detail</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-25/data-types-in-detail.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 25 – Brief on JS</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>let-and-const-keywords</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-25/let-and-const-keywords.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 25 – Brief on JS</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>conditional-statements</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-25/conditional-statements.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 25 – Brief on JS</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>generate-random-numbers-using-a-while-loop</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-25/generate-random-numbers-using-a-while-loop.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 26 – Classes</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>purpose-of-this-keyword</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-26/purpose-of-this-keyword.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 26 – Classes</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>js-class</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-26/js-class.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 26 – Classes</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>class-inheritance</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-26/class-inheritance.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 26 – Classes</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>static-methods-in-class</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-26/static-methods-in-class.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 27 – Array Sorting &amp; Mapping</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>sort-and-reverse-strings</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-27/sort-and-reverse-strings.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 27 – Array Sorting &amp; Mapping</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>sort-and-reverse-numbers</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-27/sort-and-reverse-numbers.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 27 – Array Sorting &amp; Mapping</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>map-an-array</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-27/map-an-array.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 27 – Array Sorting &amp; Mapping</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>evaluate-variables</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-27/evaluate-variables.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 28 – JS in Detail</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>type-conversion</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-28/type-conversion.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 28 – JS in Detail</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>search-and-replace-string</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-28/search-and-replace-string.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 28 – JS in Detail</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>error-handling-in-js</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-28/error-handling-in-js.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 28 – JS in Detail</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>arrow-function-in-js</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-28/arrow-function-in-js.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 29 – JSON &amp; Async</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>json-in-js</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-29/json-in-js.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 29 – JSON &amp; Async</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>callback-functions</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-29/callback-functions.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 29 – JSON &amp; Async</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>promises-in-js</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-29/promises-in-js.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 29 – JSON &amp; Async</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>async-await-in-js</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-29/async-await-in-js.html</t>
         </is>
       </c>
     </row>
@@ -2260,6 +2946,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId87"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add lesson 30 validation activities and ACP
</commit_message>
<xml_diff>
--- a/assignments_links.xlsx
+++ b/assignments_links.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2879,6 +2879,114 @@
       <c r="E88" s="7" t="inlineStr">
         <is>
           <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-29/async-await-in-js.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="12" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t>ACP</t>
+        </is>
+      </c>
+      <c r="C89" s="12" t="inlineStr">
+        <is>
+          <t>Lesson 30 – Validation in JS</t>
+        </is>
+      </c>
+      <c r="D89" s="12" t="inlineStr">
+        <is>
+          <t>validate-inputs</t>
+        </is>
+      </c>
+      <c r="E89" s="13" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/assignments/validate-inputs/validate-inputs.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 30 – Validation in JS</t>
+        </is>
+      </c>
+      <c r="D90" s="6" t="inlineStr">
+        <is>
+          <t>form-validation</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-30/form-validation.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 30 – Validation in JS</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>validation-using-api</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-30/validation-using-api.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>Lesson 30 – Validation in JS</t>
+        </is>
+      </c>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>calculator-using-js</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/abhishek-saurav/assignments_c/blob/main/m5/activities/lesson-30/calculator-using-js.html</t>
         </is>
       </c>
     </row>
@@ -2971,6 +3079,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId91"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>